<commit_message>
data: publish 2026-10-27 sampler-linked operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-10-27-182路.xlsx
+++ b/data/export/2026-10-27-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC9"/>
+  <dimension ref="A1:AC15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -441,7 +441,7 @@
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="26" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
@@ -632,32 +632,36 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:24</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>74分钟</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr"/>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -665,7 +669,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -689,17 +693,17 @@
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -709,13 +713,17 @@
       </c>
       <c r="AA2" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB2" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB2" s="2" t="inlineStr">
+        <is>
+          <t>74.0</t>
+        </is>
+      </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>2/12</t>
         </is>
       </c>
     </row>
@@ -743,32 +751,36 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:33</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>73分钟</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -776,7 +788,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -800,33 +812,37 @@
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA3" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA3" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AB3" s="2" t="inlineStr">
+        <is>
+          <t>73.0</t>
+        </is>
+      </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>1/12</t>
         </is>
       </c>
     </row>
@@ -887,7 +903,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -926,7 +942,7 @@
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA4" s="2" t="inlineStr">
@@ -937,7 +953,7 @@
       <c r="AB4" s="2" t="inlineStr"/>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/12</t>
         </is>
       </c>
     </row>
@@ -965,32 +981,36 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:53</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>78分钟</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -998,7 +1018,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1022,17 +1042,17 @@
       </c>
       <c r="W5" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X5" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y5" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z5" s="2" t="inlineStr">
@@ -1042,13 +1062,17 @@
       </c>
       <c r="AA5" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB5" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB5" s="2" t="inlineStr">
+        <is>
+          <t>78.0</t>
+        </is>
+      </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>3/12</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1133,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1159,7 +1183,7 @@
       <c r="AB6" s="2" t="inlineStr"/>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/12</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1244,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1270,7 +1294,7 @@
       <c r="AB7" s="2" t="inlineStr"/>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/12</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1355,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1381,7 +1405,7 @@
       <c r="AB8" s="2" t="inlineStr"/>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/12</t>
         </is>
       </c>
     </row>
@@ -1389,22 +1413,22 @@
       <c r="A9" s="2" t="inlineStr"/>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>沪A68870D</t>
+          <t>沪A55712D</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>07:12</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
           <t>金杨路金口路</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>07:28</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>川沙客运站</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1437,12 +1461,12 @@
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>06:02</t>
+          <t>06:42</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1456,7 +1480,7 @@
       <c r="T9" s="2" t="inlineStr"/>
       <c r="U9" s="2" t="inlineStr">
         <is>
-          <t>07:28</t>
+          <t>07:12</t>
         </is>
       </c>
       <c r="V9" s="2" t="inlineStr">
@@ -1492,7 +1516,677 @@
       <c r="AB9" s="2" t="inlineStr"/>
       <c r="AC9" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>沪A67026D</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr"/>
+      <c r="R10" s="2" t="inlineStr"/>
+      <c r="S10" s="2" t="inlineStr"/>
+      <c r="T10" s="2" t="inlineStr"/>
+      <c r="U10" s="2" t="inlineStr">
+        <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="V10" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W10" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X10" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y10" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z10" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA10" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB10" s="2" t="inlineStr"/>
+      <c r="AC10" s="2" t="inlineStr">
+        <is>
+          <t>—/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>沪A68870D</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>07:25</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="inlineStr"/>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>07:25</t>
+        </is>
+      </c>
+      <c r="V11" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y11" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z11" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA11" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB11" s="2" t="inlineStr"/>
+      <c r="AC11" s="2" t="inlineStr">
+        <is>
+          <t>—/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>沪A32899D</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>07:02</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="R12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y12" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z12" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA12" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB12" s="2" t="inlineStr"/>
+      <c r="AC12" s="2" t="inlineStr">
+        <is>
+          <t>—/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>沪A08953A</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="inlineStr"/>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y13" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z13" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA13" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB13" s="2" t="inlineStr"/>
+      <c r="AC13" s="2" t="inlineStr">
+        <is>
+          <t>—/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>沪A66513D</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>07:50</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="inlineStr"/>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>07:50</t>
+        </is>
+      </c>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y14" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA14" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB14" s="2" t="inlineStr">
+        <is>
+          <t>73.0</t>
+        </is>
+      </c>
+      <c r="AC14" s="2" t="inlineStr">
+        <is>
+          <t>1/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>沪A31073D</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z15" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA15" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB15" s="2" t="inlineStr"/>
+      <c r="AC15" s="2" t="inlineStr">
+        <is>
+          <t>—/12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: publish 2026-10-27 rolling operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-10-27-182路.xlsx
+++ b/data/export/2026-10-27-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC61"/>
+  <dimension ref="A1:AC63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -669,7 +669,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -718,7 +718,7 @@
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
-          <t>72.8</t>
+          <t>73.5</t>
         </is>
       </c>
       <c r="AC2" s="2" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AA3" s="2" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>2/13</t>
+          <t>3/13</t>
         </is>
       </c>
     </row>
@@ -907,7 +907,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -1026,7 +1026,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1070,17 +1070,17 @@
       </c>
       <c r="AA5" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
-          <t>80.0</t>
+          <t>78.4</t>
         </is>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>13/13</t>
+          <t>12/13</t>
         </is>
       </c>
     </row>
@@ -1145,7 +1145,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1260,7 +1260,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1309,7 +1309,7 @@
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
-          <t>67.0</t>
+          <t>67.5</t>
         </is>
       </c>
       <c r="AC7" s="2" t="inlineStr">
@@ -1379,7 +1379,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1498,7 +1498,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="AC10" s="2" t="inlineStr">
         <is>
-          <t>12/13</t>
+          <t>13/13</t>
         </is>
       </c>
     </row>
@@ -1732,7 +1732,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1781,12 +1781,12 @@
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
-          <t>72.3</t>
+          <t>71.3</t>
         </is>
       </c>
       <c r="AC11" s="2" t="inlineStr">
         <is>
-          <t>3/13</t>
+          <t>2/13</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>14:12</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="Z12" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA12" s="2" t="inlineStr">
@@ -2085,7 +2085,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -2124,7 +2124,7 @@
       </c>
       <c r="Z14" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AA14" s="2" t="inlineStr">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="AC14" s="2" t="inlineStr">
         <is>
-          <t>2/13</t>
+          <t>3/13</t>
         </is>
       </c>
     </row>
@@ -2200,7 +2200,7 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
@@ -2249,7 +2249,7 @@
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
-          <t>72.8</t>
+          <t>73.5</t>
         </is>
       </c>
       <c r="AC15" s="2" t="inlineStr">
@@ -2319,7 +2319,7 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -2482,17 +2482,17 @@
       </c>
       <c r="AA17" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
-          <t>80.0</t>
+          <t>78.4</t>
         </is>
       </c>
       <c r="AC17" s="2" t="inlineStr">
         <is>
-          <t>13/13</t>
+          <t>12/13</t>
         </is>
       </c>
     </row>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -2795,7 +2795,7 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -2844,7 +2844,7 @@
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
-          <t>67.0</t>
+          <t>67.5</t>
         </is>
       </c>
       <c r="AC20" s="2" t="inlineStr">
@@ -2914,7 +2914,7 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
@@ -3033,7 +3033,7 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
@@ -3206,7 +3206,7 @@
       </c>
       <c r="AC23" s="2" t="inlineStr">
         <is>
-          <t>12/13</t>
+          <t>13/13</t>
         </is>
       </c>
     </row>
@@ -3271,7 +3271,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
@@ -3320,12 +3320,12 @@
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
-          <t>72.3</t>
+          <t>71.3</t>
         </is>
       </c>
       <c r="AC24" s="2" t="inlineStr">
         <is>
-          <t>3/13</t>
+          <t>2/13</t>
         </is>
       </c>
     </row>
@@ -3390,7 +3390,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>14:12</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
@@ -3429,7 +3429,7 @@
       </c>
       <c r="Z25" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA25" s="2" t="inlineStr">
@@ -3628,7 +3628,7 @@
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
@@ -3667,7 +3667,7 @@
       </c>
       <c r="Z27" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AA27" s="2" t="inlineStr">
@@ -3682,7 +3682,7 @@
       </c>
       <c r="AC27" s="2" t="inlineStr">
         <is>
-          <t>2/13</t>
+          <t>3/13</t>
         </is>
       </c>
     </row>
@@ -3747,7 +3747,7 @@
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
@@ -3796,7 +3796,7 @@
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
-          <t>72.8</t>
+          <t>73.5</t>
         </is>
       </c>
       <c r="AC28" s="2" t="inlineStr">
@@ -3866,7 +3866,7 @@
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
@@ -3985,7 +3985,7 @@
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
@@ -4029,17 +4029,17 @@
       </c>
       <c r="AA30" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
-          <t>80.0</t>
+          <t>78.4</t>
         </is>
       </c>
       <c r="AC30" s="2" t="inlineStr">
         <is>
-          <t>13/13</t>
+          <t>12/13</t>
         </is>
       </c>
     </row>
@@ -4223,7 +4223,7 @@
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr">
@@ -4342,7 +4342,7 @@
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P33" s="2" t="inlineStr">
@@ -4461,7 +4461,7 @@
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P34" s="2" t="inlineStr">
@@ -4580,7 +4580,7 @@
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P35" s="2" t="inlineStr">
@@ -4629,12 +4629,12 @@
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
-          <t>72.3</t>
+          <t>71.3</t>
         </is>
       </c>
       <c r="AC35" s="2" t="inlineStr">
         <is>
-          <t>3/13</t>
+          <t>2/13</t>
         </is>
       </c>
     </row>
@@ -4699,7 +4699,7 @@
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>14:12</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
@@ -4738,7 +4738,7 @@
       </c>
       <c r="Z36" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA36" s="2" t="inlineStr">
@@ -4818,7 +4818,7 @@
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P37" s="2" t="inlineStr">
@@ -4857,7 +4857,7 @@
       </c>
       <c r="Z37" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AA37" s="2" t="inlineStr">
@@ -4872,7 +4872,7 @@
       </c>
       <c r="AC37" s="2" t="inlineStr">
         <is>
-          <t>2/13</t>
+          <t>3/13</t>
         </is>
       </c>
     </row>
@@ -5056,7 +5056,7 @@
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P39" s="2" t="inlineStr">
@@ -5294,7 +5294,7 @@
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P41" s="2" t="inlineStr">
@@ -5413,7 +5413,7 @@
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P42" s="2" t="inlineStr">
@@ -5586,7 +5586,7 @@
       </c>
       <c r="AC43" s="2" t="inlineStr">
         <is>
-          <t>12/13</t>
+          <t>13/13</t>
         </is>
       </c>
     </row>
@@ -5651,7 +5651,7 @@
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>14:12</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P44" s="2" t="inlineStr">
@@ -5690,7 +5690,7 @@
       </c>
       <c r="Z44" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA44" s="2" t="inlineStr">
@@ -5770,7 +5770,7 @@
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P45" s="2" t="inlineStr">
@@ -5819,7 +5819,7 @@
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
-          <t>72.8</t>
+          <t>73.5</t>
         </is>
       </c>
       <c r="AC45" s="2" t="inlineStr">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P47" s="2" t="inlineStr">
@@ -6052,17 +6052,17 @@
       </c>
       <c r="AA47" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
-          <t>80.0</t>
+          <t>78.4</t>
         </is>
       </c>
       <c r="AC47" s="2" t="inlineStr">
         <is>
-          <t>13/13</t>
+          <t>12/13</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P49" s="2" t="inlineStr">
@@ -6419,7 +6419,7 @@
       </c>
       <c r="AC50" s="2" t="inlineStr">
         <is>
-          <t>12/13</t>
+          <t>13/13</t>
         </is>
       </c>
     </row>
@@ -6457,24 +6457,24 @@
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>15:38</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>73分钟</t>
+          <t>70分钟</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr"/>
       <c r="K51" s="2" t="inlineStr"/>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
         </is>
       </c>
       <c r="M51" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N51" s="2" t="inlineStr">
@@ -6484,7 +6484,7 @@
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P51" s="2" t="inlineStr">
@@ -6533,12 +6533,12 @@
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
-          <t>72.3</t>
+          <t>71.3</t>
         </is>
       </c>
       <c r="AC51" s="2" t="inlineStr">
         <is>
-          <t>3/13</t>
+          <t>2/13</t>
         </is>
       </c>
     </row>
@@ -6576,12 +6576,12 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>15:53</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>73分钟</t>
+          <t>76分钟</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr"/>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P52" s="2" t="inlineStr">
@@ -6652,7 +6652,7 @@
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
-          <t>72.8</t>
+          <t>73.5</t>
         </is>
       </c>
       <c r="AC52" s="2" t="inlineStr">
@@ -6695,12 +6695,12 @@
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>66分钟</t>
+          <t>67分钟</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr"/>
@@ -6722,7 +6722,7 @@
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P53" s="2" t="inlineStr">
@@ -6771,7 +6771,7 @@
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
-          <t>67.0</t>
+          <t>67.5</t>
         </is>
       </c>
       <c r="AC53" s="2" t="inlineStr">
@@ -6804,32 +6804,36 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>16:12</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>72分钟</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr"/>
       <c r="K54" s="2" t="inlineStr"/>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M54" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±4分钟</t>
+        </is>
+      </c>
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="N54" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -6837,7 +6841,7 @@
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P54" s="2" t="inlineStr">
@@ -6861,17 +6865,17 @@
       </c>
       <c r="W54" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X54" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y54" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z54" s="2" t="inlineStr">
@@ -6881,17 +6885,17 @@
       </c>
       <c r="AA54" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
-          <t>80.0</t>
+          <t>78.4</t>
         </is>
       </c>
       <c r="AC54" s="2" t="inlineStr">
         <is>
-          <t>13/13</t>
+          <t>12/13</t>
         </is>
       </c>
     </row>
@@ -6952,7 +6956,7 @@
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P55" s="2" t="inlineStr">
@@ -6991,7 +6995,7 @@
       </c>
       <c r="Z55" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AA55" s="2" t="inlineStr">
@@ -7006,7 +7010,7 @@
       </c>
       <c r="AC55" s="2" t="inlineStr">
         <is>
-          <t>2/13</t>
+          <t>3/13</t>
         </is>
       </c>
     </row>
@@ -7067,7 +7071,7 @@
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P56" s="2" t="inlineStr">
@@ -7182,7 +7186,7 @@
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P57" s="2" t="inlineStr">
@@ -7297,7 +7301,7 @@
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P58" s="2" t="inlineStr">
@@ -7412,7 +7416,7 @@
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P59" s="2" t="inlineStr">
@@ -7461,12 +7465,12 @@
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
-          <t>72.3</t>
+          <t>71.3</t>
         </is>
       </c>
       <c r="AC59" s="2" t="inlineStr">
         <is>
-          <t>3/13</t>
+          <t>2/13</t>
         </is>
       </c>
     </row>
@@ -7527,7 +7531,7 @@
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P60" s="2" t="inlineStr">
@@ -7642,7 +7646,7 @@
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="P61" s="2" t="inlineStr">
@@ -7691,12 +7695,242 @@
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
-          <t>67.0</t>
+          <t>67.5</t>
         </is>
       </c>
       <c r="AC61" s="2" t="inlineStr">
         <is>
           <t>1/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr"/>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>沪A32899D</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>16:12</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr"/>
+      <c r="K62" s="2" t="inlineStr"/>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M62" s="2" t="inlineStr"/>
+      <c r="N62" s="2" t="inlineStr">
+        <is>
+          <t>07:02</t>
+        </is>
+      </c>
+      <c r="O62" s="2" t="inlineStr">
+        <is>
+          <t>15:42</t>
+        </is>
+      </c>
+      <c r="P62" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q62" s="2" t="inlineStr"/>
+      <c r="R62" s="2" t="inlineStr"/>
+      <c r="S62" s="2" t="inlineStr"/>
+      <c r="T62" s="2" t="inlineStr"/>
+      <c r="U62" s="2" t="inlineStr">
+        <is>
+          <t>16:12</t>
+        </is>
+      </c>
+      <c r="V62" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W62" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X62" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y62" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z62" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AA62" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AB62" s="2" t="inlineStr">
+        <is>
+          <t>78.2</t>
+        </is>
+      </c>
+      <c r="AC62" s="2" t="inlineStr">
+        <is>
+          <t>11/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr"/>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>沪A66513D</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr"/>
+      <c r="K63" s="2" t="inlineStr"/>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M63" s="2" t="inlineStr"/>
+      <c r="N63" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O63" s="2" t="inlineStr">
+        <is>
+          <t>15:42</t>
+        </is>
+      </c>
+      <c r="P63" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q63" s="2" t="inlineStr"/>
+      <c r="R63" s="2" t="inlineStr"/>
+      <c r="S63" s="2" t="inlineStr"/>
+      <c r="T63" s="2" t="inlineStr"/>
+      <c r="U63" s="2" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="V63" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W63" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X63" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y63" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z63" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AA63" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AB63" s="2" t="inlineStr">
+        <is>
+          <t>72.0</t>
+        </is>
+      </c>
+      <c r="AC63" s="2" t="inlineStr">
+        <is>
+          <t>3/13</t>
         </is>
       </c>
     </row>

</xml_diff>